<commit_message>
C8 (RKB): the pre-reform eps is 70% of the minimum pension, so getEps reads the first formal quartile by label in both Argentine modules (it read the second by position); gamma0 = 0.32/0.68 in data/ArgentinaTest.xlsx so informal households are 32% of all; docstrings, data/README, TODO C8 in progress, module and root logs. The Argentine arm re-solves as logs/finalRunC8/runArg.cmd; results and the paper's numbers follow when it is read
</commit_message>
<xml_diff>
--- a/data/ArgentinaTest.xlsx
+++ b/data/ArgentinaTest.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sxj477\Documents\GitHub\SSDclaude\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{225BBA8B-8297-498E-9CD0-D4716653730B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{975FA60E-BAF6-4B46-B858-214F8F7B75C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{D3C4F84A-0E01-44C3-A15D-A44758EFE8C0}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" activeTab="2" xr2:uid="{D3C4F84A-0E01-44C3-A15D-A44758EFE8C0}"/>
   </bookViews>
   <sheets>
     <sheet name="population" sheetId="1" r:id="rId1"/>
@@ -467,12 +467,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D43B1461-40F3-4621-A383-5FE9A849ADE2}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.1328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -480,7 +480,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A2">
         <v>1920</v>
       </c>
@@ -489,7 +489,7 @@
         <v>1.645994618709391</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A3">
         <v>1950</v>
       </c>
@@ -498,7 +498,7 @@
         <v>1.645994618709391</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A4">
         <v>1980</v>
       </c>
@@ -506,7 +506,7 @@
         <v>1.645994618709391</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A5">
         <v>2010</v>
       </c>
@@ -514,7 +514,7 @@
         <v>1.473985729446017</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A6">
         <v>2040</v>
       </c>
@@ -522,7 +522,7 @@
         <v>1.1581292709104491</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A7">
         <v>2070</v>
       </c>
@@ -530,7 +530,7 @@
         <v>0.96408919724182562</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.75">
       <c r="A8">
         <v>2100</v>
       </c>
@@ -547,14 +547,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CE76B0EF-4908-4CB2-98A8-B49EE220FB32}">
   <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="2" max="2" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.40625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.1328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>3</v>
       </c>
@@ -574,12 +574,12 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.75">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2">
-        <v>0.32</v>
+        <v>0.47058823529411764</v>
       </c>
       <c r="C2">
         <v>0.66416666700000004</v>
@@ -594,7 +594,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.75">
       <c r="A3">
         <v>1</v>
       </c>
@@ -614,7 +614,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.75">
       <c r="A4">
         <v>2</v>
       </c>
@@ -634,7 +634,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.75">
       <c r="A5">
         <v>3</v>
       </c>
@@ -654,7 +654,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.75">
       <c r="A6">
         <v>4</v>
       </c>
@@ -682,19 +682,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{11E48DC5-CA22-4A6E-BD10-69F2BD6158FF}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.1328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="24.140625" customWidth="1"/>
-    <col min="8" max="8" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.86328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.1328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.40625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.1328125" customWidth="1"/>
+    <col min="8" max="8" width="17.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>7</v>
       </c>
@@ -720,7 +720,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.75">
       <c r="A2">
         <v>2010</v>
       </c>

</xml_diff>